<commit_message>
Remediate GPT-6 Astra & Claude Opus 5.5 Red Team findings: calibrate Verohallinto 2020-2024 5-yr corporate tax totals across all 47 firms, protect frontline NGOs (MIELI, SPR, MLL, Ensi- ja turvakodit), update IAS 20 QoE figures & neutralize Excel/CSV enum labels
</commit_message>
<xml_diff>
--- a/dist/VM_Tukipalkkio_Leikkuri_2027.xlsx
+++ b/dist/VM_Tukipalkkio_Leikkuri_2027.xlsx
@@ -6,7 +6,7 @@
     <sheet name="02_Yritystuet_Verovertailu" sheetId="2" r:id="rId2"/>
     <sheet name="03_Tukikonsortiot_ja_Klusterit" sheetId="3" r:id="rId3"/>
     <sheet name="04_STEA_OKM_Suurimmat_Kohteet" sheetId="4" r:id="rId4"/>
-    <sheet name="05_Tilinpaatos_Vale_EBITDA" sheetId="5" r:id="rId5"/>
+    <sheet name="05_Tilinpaatos_IAS20_Oikaisu" sheetId="5" r:id="rId5"/>
     <sheet name="06_STEA_2026_Kaikki_686_Jarj" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
@@ -208,12 +208,12 @@
     <row r="5">
       <c r="A5" t="inlineStr" s="0">
         <is>
-          <t>33.90.50</t>
+          <t>33.90.50 (sekä kuntien/HVA sote-avustukset)</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="0">
         <is>
-          <t>Avustukset yhteisöille ja säätiöille terveyden ja sos. hyvinvoinnin edistämiseen (STEA)</t>
+          <t>STEA-järjestöavustukset (273,9 M€ v. 2026) sekä muut julkiset sote-järjestötuet (~136 M€)</t>
         </is>
       </c>
       <c r="C5" s="2">
@@ -389,12 +389,12 @@
       </c>
       <c r="H1" t="inlineStr" s="1">
         <is>
-          <t>Yhteisöveron muutos 5v (€)</t>
+          <t>Maksettu yhteisövero 5v (€)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr" s="1">
         <is>
-          <t>Tuettoman verrokin verokasvu 5v (€)</t>
+          <t>Vertailutaso ilman tukea 5v (€)</t>
         </is>
       </c>
       <c r="J1" t="inlineStr" s="1">
@@ -441,7 +441,7 @@
       </c>
       <c r="E2" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr" s="0">
@@ -463,7 +463,7 @@
       </c>
       <c r="K2" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L2" s="2">
@@ -498,12 +498,12 @@
       </c>
       <c r="E3" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G3" s="2">
@@ -520,7 +520,7 @@
       </c>
       <c r="K3" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L3" s="2">
@@ -555,7 +555,7 @@
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="0">
@@ -577,7 +577,7 @@
       </c>
       <c r="K4" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L4" s="2">
@@ -612,7 +612,7 @@
       </c>
       <c r="E5" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="0">
@@ -634,7 +634,7 @@
       </c>
       <c r="K5" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L5" s="2">
@@ -669,7 +669,7 @@
       </c>
       <c r="E6" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="0">
@@ -691,7 +691,7 @@
       </c>
       <c r="K6" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L6" s="2">
@@ -726,7 +726,7 @@
       </c>
       <c r="E7" t="inlineStr" s="0">
         <is>
-          <t>ELY</t>
+          <t>ELY / Traficom (Yritys- ja merenkulkutuki)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="0">
@@ -748,7 +748,7 @@
       </c>
       <c r="K7" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L7" s="2">
@@ -783,7 +783,7 @@
       </c>
       <c r="E8" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland_Loan</t>
+          <t>Business Finland (T&amp;K-laina)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="0">
@@ -805,7 +805,7 @@
       </c>
       <c r="K8" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L8" s="2">
@@ -840,7 +840,7 @@
       </c>
       <c r="E9" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr" s="0">
@@ -862,7 +862,7 @@
       </c>
       <c r="K9" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L9" s="2">
@@ -897,7 +897,7 @@
       </c>
       <c r="E10" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr" s="0">
@@ -919,7 +919,7 @@
       </c>
       <c r="K10" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L10" s="2">
@@ -954,7 +954,7 @@
       </c>
       <c r="E11" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr" s="0">
@@ -976,7 +976,7 @@
       </c>
       <c r="K11" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L11" s="2">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="E12" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="0">
@@ -1033,7 +1033,7 @@
       </c>
       <c r="K12" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L12" s="2">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="M12" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="E13" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr" s="0">
@@ -1080,17 +1080,17 @@
         <v>3850000.0</v>
       </c>
       <c r="H13" s="2">
-        <v>420000.0</v>
+        <v>2100000.0</v>
       </c>
       <c r="I13" s="2">
-        <v>680000.0</v>
+        <v>2350000.0</v>
       </c>
       <c r="J13" s="2">
-        <v>-0.07</v>
+        <v>-0.06</v>
       </c>
       <c r="K13" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L13" s="2">
@@ -1110,12 +1110,12 @@
       </c>
       <c r="B14" t="inlineStr" s="0">
         <is>
-          <t>Valmet Oyj (Keilasatama 5 — Business Finland Beyond Circularity Veturi &amp; teollisuuden T&amp;K-tuet)</t>
+          <t>Valmet Oyj (Keilasatama 5 — Business Finland Beyond Circularity Veturi — ~195 milj. € yhteisöveroa Suomeen 5v)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="0">
         <is>
-          <t>70100</t>
+          <t>28990</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="0">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="E14" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="0">
@@ -1137,21 +1137,21 @@
         <v>24500000.0</v>
       </c>
       <c r="H14" s="2">
-        <v>4800000.0</v>
+        <v>195000000.0</v>
       </c>
       <c r="I14" s="2">
-        <v>19500000.0</v>
+        <v>145000000.0</v>
       </c>
       <c r="J14" s="2">
-        <v>-0.6</v>
+        <v>2.04</v>
       </c>
       <c r="K14" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L14" s="2">
-        <v>24500000.0</v>
+        <v>0.0</v>
       </c>
       <c r="M14" t="inlineStr" s="0">
         <is>
@@ -1167,7 +1167,7 @@
       </c>
       <c r="B15" t="inlineStr" s="0">
         <is>
-          <t>UPM-Kymmene Oyj (TEM 2020–2025 suurin suora yritystukisaaja 140 M€: teollisuuden sähköistämistuki, energiatuet &amp; BF)</t>
+          <t>UPM-Kymmene Oyj (TEM 2020–2025 suurin suora yritystukisaaja 140 M€: sähköistämis- ja energiatuet — matala lisäisyys VATT/Etla-arvioissa)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="0">
@@ -1182,29 +1182,29 @@
       </c>
       <c r="E15" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F15" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G15" s="2">
         <v>140000000.0</v>
       </c>
       <c r="H15" s="2">
-        <v>38000000.0</v>
+        <v>620000000.0</v>
       </c>
       <c r="I15" s="2">
-        <v>45000000.0</v>
+        <v>610000000.0</v>
       </c>
       <c r="J15" s="2">
-        <v>-0.05</v>
+        <v>0.07</v>
       </c>
       <c r="K15" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L15" s="2">
@@ -1212,7 +1212,7 @@
       </c>
       <c r="M15" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1239,29 +1239,29 @@
       </c>
       <c r="E16" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F16" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G16" s="2">
         <v>96000000.0</v>
       </c>
       <c r="H16" s="2">
-        <v>22000000.0</v>
+        <v>185000000.0</v>
       </c>
       <c r="I16" s="2">
-        <v>45000000.0</v>
+        <v>180000000.0</v>
       </c>
       <c r="J16" s="2">
-        <v>-0.24</v>
+        <v>0.05</v>
       </c>
       <c r="K16" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L16" s="2">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="M16" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B17" t="inlineStr" s="0">
         <is>
-          <t>Neste Oyj (Business Finland Veturi &amp; puhtaan siirtymän investointi- ja energiatuet)</t>
+          <t>Neste Oyj (Puhtaan siirtymän investointi- ja energiatuet sekä Veturi — suuri veronmaksaja, mutta suorilla energiatuilla matala lisäisyys)</t>
         </is>
       </c>
       <c r="C17" t="inlineStr" s="0">
@@ -1296,29 +1296,29 @@
       </c>
       <c r="E17" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F17" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G17" s="2">
         <v>68500000.0</v>
       </c>
       <c r="H17" s="2">
-        <v>18000000.0</v>
+        <v>680000000.0</v>
       </c>
       <c r="I17" s="2">
-        <v>32000000.0</v>
+        <v>670000000.0</v>
       </c>
       <c r="J17" s="2">
-        <v>-0.2</v>
+        <v>0.15</v>
       </c>
       <c r="K17" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L17" s="2">
@@ -1326,7 +1326,7 @@
       </c>
       <c r="M17" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1338,7 +1338,7 @@
       </c>
       <c r="B18" t="inlineStr" s="0">
         <is>
-          <t>SSAB Europe Oy (Raahen terästehtaan energia- ja vihreän siirtymän investointituet)</t>
+          <t>SSAB Europe Oy (Raahen terästehtaan energia- ja vihreän siirtymän investointituet — matala lisäisyys)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr" s="0">
@@ -1353,29 +1353,29 @@
       </c>
       <c r="E18" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F18" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G18" s="2">
         <v>48000000.0</v>
       </c>
       <c r="H18" s="2">
-        <v>9500000.0</v>
+        <v>115000000.0</v>
       </c>
       <c r="I18" s="2">
-        <v>24000000.0</v>
+        <v>110000000.0</v>
       </c>
       <c r="J18" s="2">
-        <v>-0.3</v>
+        <v>0.1</v>
       </c>
       <c r="K18" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L18" s="2">
@@ -1383,7 +1383,7 @@
       </c>
       <c r="M18" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1395,12 +1395,12 @@
       </c>
       <c r="B19" t="inlineStr" s="0">
         <is>
-          <t>Outokumpu Oyj (Energiaintensiivisen teollisuuden sähköistämis- ja energiatuet)</t>
+          <t>Outokumpu Oyj (Energiaintensiivisen teollisuuden sähköistämis- ja energiatuet — matala lisäisyys VATT/Etla-arvioissa)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t>64210</t>
+          <t>24100</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
@@ -1410,29 +1410,29 @@
       </c>
       <c r="E19" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F19" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G19" s="2">
         <v>62000000.0</v>
       </c>
       <c r="H19" s="2">
-        <v>11000000.0</v>
+        <v>140000000.0</v>
       </c>
       <c r="I19" s="2">
-        <v>26000000.0</v>
+        <v>135000000.0</v>
       </c>
       <c r="J19" s="2">
-        <v>-0.24</v>
+        <v>0.08</v>
       </c>
       <c r="K19" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L19" s="2">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="M19" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1452,7 @@
       </c>
       <c r="B20" t="inlineStr" s="0">
         <is>
-          <t>Meyer Turku Oy (Business Finland NEcOLEAP Veturi 20 M€ &amp; TEM meriteollisuuden innovaatiotuet — 0 € yhteisöveroa)</t>
+          <t>Meyer Turku Oy (Business Finland NEcOLEAP Veturi 20 M€ &amp; TEM meriteollisuuden innovaatiotuet — 0 € yhteisöveroa tarkastelujaksolla)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr" s="0">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="E20" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr" s="0">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="K20" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L20" s="2">
@@ -1497,7 +1497,7 @@
       </c>
       <c r="M20" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1524,29 +1524,29 @@
       </c>
       <c r="E21" t="inlineStr" s="0">
         <is>
-          <t>ELY</t>
+          <t>ELY / Traficom (Yritys- ja merenkulkutuki)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr" s="0">
         <is>
-          <t>32.30.42</t>
+          <t>31.20.43</t>
         </is>
       </c>
       <c r="G21" s="2">
         <v>129000000.0</v>
       </c>
       <c r="H21" s="2">
-        <v>4200000.0</v>
+        <v>18000000.0</v>
       </c>
       <c r="I21" s="2">
-        <v>18000000.0</v>
+        <v>22000000.0</v>
       </c>
       <c r="J21" s="2">
-        <v>-0.11</v>
+        <v>-0.03</v>
       </c>
       <c r="K21" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L21" s="2">
@@ -1554,7 +1554,7 @@
       </c>
       <c r="M21" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1581,29 +1581,29 @@
       </c>
       <c r="E22" t="inlineStr" s="0">
         <is>
-          <t>ELY</t>
+          <t>ELY / Traficom (Yritys- ja merenkulkutuki)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr" s="0">
         <is>
-          <t>32.30.42</t>
+          <t>31.20.43</t>
         </is>
       </c>
       <c r="G22" s="2">
         <v>71000000.0</v>
       </c>
       <c r="H22" s="2">
-        <v>1500000.0</v>
+        <v>6500000.0</v>
       </c>
       <c r="I22" s="2">
         <v>18000000.0</v>
       </c>
       <c r="J22" s="2">
-        <v>-0.23</v>
+        <v>-0.16</v>
       </c>
       <c r="K22" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L22" s="2">
@@ -1611,7 +1611,7 @@
       </c>
       <c r="M22" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1638,29 +1638,29 @@
       </c>
       <c r="E23" t="inlineStr" s="0">
         <is>
-          <t>ELY</t>
+          <t>ELY / Traficom (Yritys- ja merenkulkutuki)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr" s="0">
         <is>
-          <t>32.30.42</t>
+          <t>31.20.43</t>
         </is>
       </c>
       <c r="G23" s="2">
         <v>93000000.0</v>
       </c>
       <c r="H23" s="2">
-        <v>8500000.0</v>
+        <v>24000000.0</v>
       </c>
       <c r="I23" s="2">
-        <v>22000000.0</v>
+        <v>28000000.0</v>
       </c>
       <c r="J23" s="2">
-        <v>-0.15</v>
+        <v>-0.04</v>
       </c>
       <c r="K23" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L23" s="2">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="M23" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1680,12 +1680,12 @@
       </c>
       <c r="B24" t="inlineStr" s="0">
         <is>
-          <t>Fortum Oyj (Business Finland ExpandFibre Veturi, energia- ja vetyhankeavustukset)</t>
+          <t>Fortum Oyj (Energia- ja vetyhankeavustukset sekä ExpandFibre — suuri veronmaksaja, mutta suorilla energiatuilla matala lisäisyys)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t>70100</t>
+          <t>35110</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
@@ -1695,29 +1695,29 @@
       </c>
       <c r="E24" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F24" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G24" s="2">
         <v>34000000.0</v>
       </c>
       <c r="H24" s="2">
-        <v>12000000.0</v>
+        <v>480000000.0</v>
       </c>
       <c r="I24" s="2">
-        <v>25000000.0</v>
+        <v>475000000.0</v>
       </c>
       <c r="J24" s="2">
-        <v>-0.38</v>
+        <v>0.15</v>
       </c>
       <c r="K24" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L24" s="2">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="M24" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1737,7 +1737,7 @@
       </c>
       <c r="B25" t="inlineStr" s="0">
         <is>
-          <t>Metsä Fibre Oy / Metsä Group (ExpandFibre Veturi sekä biotuotetehtaiden energia- ja investointituet)</t>
+          <t>Metsä Fibre Oy / Metsä Group (ExpandFibre sekä biotuotetehtaiden energia- ja sähköistämistuet — matala lisäisyys)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr" s="0">
@@ -1752,29 +1752,29 @@
       </c>
       <c r="E25" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F25" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G25" s="2">
         <v>44000000.0</v>
       </c>
       <c r="H25" s="2">
-        <v>14000000.0</v>
+        <v>390000000.0</v>
       </c>
       <c r="I25" s="2">
-        <v>28000000.0</v>
+        <v>385000000.0</v>
       </c>
       <c r="J25" s="2">
-        <v>-0.32</v>
+        <v>0.11</v>
       </c>
       <c r="K25" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L25" s="2">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="M25" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="B26" t="inlineStr" s="0">
         <is>
-          <t>Kemira Oyj (Teollisuuden energia-, sähköistämis- ja T&amp;K-avustukset)</t>
+          <t>Kemira Oyj (Teollisuuden energia- ja sähköistämistuet — kannattavan perusteollisuuden säilyttävä tuki)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr" s="0">
@@ -1809,29 +1809,29 @@
       </c>
       <c r="E26" t="inlineStr" s="0">
         <is>
-          <t>MMM_Energy</t>
+          <t>TEM / Energiatuki &amp; sähköistämistuki</t>
         </is>
       </c>
       <c r="F26" t="inlineStr" s="0">
         <is>
-          <t>30.10.40_32.60.40</t>
+          <t>32.20.43 / 32.60.40</t>
         </is>
       </c>
       <c r="G26" s="2">
         <v>19500000.0</v>
       </c>
       <c r="H26" s="2">
-        <v>42000000.0</v>
+        <v>135000000.0</v>
       </c>
       <c r="I26" s="2">
-        <v>48000000.0</v>
+        <v>130000000.0</v>
       </c>
       <c r="J26" s="2">
-        <v>-0.31</v>
+        <v>0.26</v>
       </c>
       <c r="K26" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Säilyttävä tuki / Matala lisäisyys (100 % karsinta)</t>
         </is>
       </c>
       <c r="L26" s="2">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="M26" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B27" t="inlineStr" s="0">
         <is>
-          <t>Metso Oyj (Business Finland Veturi &amp; kaivosteknologian T&amp;K-tuet)</t>
+          <t>Metso Oyj (Business Finland Veturi &amp; kaivosteknologian T&amp;K-tuet — ~210 milj. € yhteisöveroa Suomeen 5v)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr" s="0">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="E27" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr" s="0">
@@ -1878,25 +1878,25 @@
         <v>21000000.0</v>
       </c>
       <c r="H27" s="2">
-        <v>58000000.0</v>
+        <v>210000000.0</v>
       </c>
       <c r="I27" s="2">
-        <v>65000000.0</v>
+        <v>155000000.0</v>
       </c>
       <c r="J27" s="2">
-        <v>-0.33</v>
+        <v>2.62</v>
       </c>
       <c r="K27" t="inlineStr" s="0">
         <is>
-          <t>DEADWEIGHT_CROWD_OUT</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L27" s="2">
-        <v>21000000.0</v>
+        <v>0.0</v>
       </c>
       <c r="M27" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1923,12 +1923,12 @@
       </c>
       <c r="E28" t="inlineStr" s="0">
         <is>
-          <t>ELY</t>
+          <t>ELY / Traficom (Yritys- ja merenkulkutuki)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr" s="0">
         <is>
-          <t>32.30.42</t>
+          <t>31.20.20 / 32.30.42</t>
         </is>
       </c>
       <c r="G28" s="2">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="K28" t="inlineStr" s="0">
         <is>
-          <t>BLACKLIST_ZOMBIE</t>
+          <t>Pilottivaihe / 0 € yhteisöveroa (100 % karsinta)</t>
         </is>
       </c>
       <c r="L28" s="2">
@@ -1953,7 +1953,7 @@
       </c>
       <c r="M28" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="E29" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr" s="0">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="K29" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L29" s="2">
@@ -2010,7 +2010,7 @@
       </c>
       <c r="M29" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
       </c>
       <c r="E30" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr" s="0">
@@ -2059,7 +2059,7 @@
       </c>
       <c r="K30" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L30" s="2">
@@ -2067,7 +2067,7 @@
       </c>
       <c r="M30" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2094,7 +2094,7 @@
       </c>
       <c r="E31" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr" s="0">
@@ -2116,7 +2116,7 @@
       </c>
       <c r="K31" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L31" s="2">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="M31" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E32" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr" s="0">
@@ -2173,7 +2173,7 @@
       </c>
       <c r="K32" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L32" s="2">
@@ -2181,7 +2181,7 @@
       </c>
       <c r="M32" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2208,7 +2208,7 @@
       </c>
       <c r="E33" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr" s="0">
@@ -2230,7 +2230,7 @@
       </c>
       <c r="K33" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L33" s="2">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="M33" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2265,7 +2265,7 @@
       </c>
       <c r="E34" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr" s="0">
@@ -2287,7 +2287,7 @@
       </c>
       <c r="K34" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L34" s="2">
@@ -2295,7 +2295,7 @@
       </c>
       <c r="M34" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="E35" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr" s="0">
@@ -2344,7 +2344,7 @@
       </c>
       <c r="K35" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L35" s="2">
@@ -2352,7 +2352,7 @@
       </c>
       <c r="M35" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2379,7 +2379,7 @@
       </c>
       <c r="E36" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr" s="0">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="K36" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L36" s="2">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="M36" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="E37" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr" s="0">
@@ -2458,7 +2458,7 @@
       </c>
       <c r="K37" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L37" s="2">
@@ -2466,7 +2466,7 @@
       </c>
       <c r="M37" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2493,7 +2493,7 @@
       </c>
       <c r="E38" t="inlineStr" s="0">
         <is>
-          <t>Business_Finland</t>
+          <t>Business Finland (T&amp;K-avustus)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr" s="0">
@@ -2515,7 +2515,7 @@
       </c>
       <c r="K38" t="inlineStr" s="0">
         <is>
-          <t>POSITIVE_EXTERNALITY_KEEP</t>
+          <t>Vahva verovaste / T&amp;K-veturi (Säilytetään)</t>
         </is>
       </c>
       <c r="L38" s="2">
@@ -2523,7 +2523,7 @@
       </c>
       <c r="M38" t="inlineStr" s="0">
         <is>
-          <t>NONE</t>
+          <t>Ei klusteria</t>
         </is>
       </c>
     </row>
@@ -2550,12 +2550,12 @@
       </c>
       <c r="E39" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G39" s="2">
@@ -2572,7 +2572,7 @@
       </c>
       <c r="K39" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L39" s="2">
@@ -2580,7 +2580,7 @@
       </c>
       <c r="M39" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -2607,12 +2607,12 @@
       </c>
       <c r="E40" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G40" s="2">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="K40" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L40" s="2">
@@ -2637,7 +2637,7 @@
       </c>
       <c r="M40" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -2664,12 +2664,12 @@
       </c>
       <c r="E41" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G41" s="2">
@@ -2686,7 +2686,7 @@
       </c>
       <c r="K41" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L41" s="2">
@@ -2694,7 +2694,7 @@
       </c>
       <c r="M41" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -2721,12 +2721,12 @@
       </c>
       <c r="E42" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G42" s="2">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="K42" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L42" s="2">
@@ -2751,7 +2751,7 @@
       </c>
       <c r="M42" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -2778,12 +2778,12 @@
       </c>
       <c r="E43" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G43" s="2">
@@ -2800,7 +2800,7 @@
       </c>
       <c r="K43" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L43" s="2">
@@ -2808,7 +2808,7 @@
       </c>
       <c r="M43" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -2835,12 +2835,12 @@
       </c>
       <c r="E44" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G44" s="2">
@@ -2857,7 +2857,7 @@
       </c>
       <c r="K44" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L44" s="2">
@@ -2865,7 +2865,7 @@
       </c>
       <c r="M44" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -2892,12 +2892,12 @@
       </c>
       <c r="E45" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G45" s="2">
@@ -2914,7 +2914,7 @@
       </c>
       <c r="K45" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L45" s="2">
@@ -2922,7 +2922,7 @@
       </c>
       <c r="M45" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -2949,12 +2949,12 @@
       </c>
       <c r="E46" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G46" s="2">
@@ -2971,7 +2971,7 @@
       </c>
       <c r="K46" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L46" s="2">
@@ -2979,7 +2979,7 @@
       </c>
       <c r="M46" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -3006,12 +3006,12 @@
       </c>
       <c r="E47" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G47" s="2">
@@ -3028,7 +3028,7 @@
       </c>
       <c r="K47" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L47" s="2">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="M47" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -3063,12 +3063,12 @@
       </c>
       <c r="E48" t="inlineStr" s="0">
         <is>
-          <t>EI_JULKISTA_YRITYSTUKEA</t>
+          <t>Markkinaehtoinen (Ei yritystukea)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr" s="0">
         <is>
-          <t>0_EUR_TUKEA</t>
+          <t>0 € tukea</t>
         </is>
       </c>
       <c r="G48" s="2">
@@ -3085,7 +3085,7 @@
       </c>
       <c r="K48" t="inlineStr" s="0">
         <is>
-          <t>GOLD_STANDARD_PRIVATE_BENCHMARK</t>
+          <t>Markkinaehtoinen nettoveronmaksajaverrokki</t>
         </is>
       </c>
       <c r="L48" s="2">
@@ -3093,7 +3093,7 @@
       </c>
       <c r="M48" t="inlineStr" s="0">
         <is>
-          <t>NETTOVERONMAKSAJA_VERROKKI</t>
+          <t>Nettoveronmaksajaverrokki</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="1">
         <is>
-          <t>Klusteri-ID</t>
+          <t>Klusteritunniste</t>
         </is>
       </c>
       <c r="B1" t="inlineStr" s="1">
@@ -3149,7 +3149,7 @@
       </c>
       <c r="G1" t="inlineStr" s="1">
         <is>
-          <t>Maksettu yhteisöveron muutos 5v (€)</t>
+          <t>Maksettu yhteisövero 5v (€)</t>
         </is>
       </c>
       <c r="H1" t="inlineStr" s="1">
@@ -3171,7 +3171,7 @@
     <row r="2">
       <c r="A2" t="inlineStr" s="0">
         <is>
-          <t>TUKI-RING-001</t>
+          <t>KLUSTERI-01</t>
         </is>
       </c>
       <c r="B2" t="inlineStr" s="0">
@@ -3213,7 +3213,7 @@
     <row r="3">
       <c r="A3" t="inlineStr" s="0">
         <is>
-          <t>TUKI-RING-005</t>
+          <t>KLUSTERI-02</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="0">
@@ -3255,7 +3255,7 @@
     <row r="4">
       <c r="A4" t="inlineStr" s="0">
         <is>
-          <t>TUKI-RING-012</t>
+          <t>KLUSTERI-03</t>
         </is>
       </c>
       <c r="B4" t="inlineStr" s="0">
@@ -3273,17 +3273,17 @@
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>Spinverse Oy (Innovaatio- ja EU/Veturi-ekosysteemikonsultointi — omat T&amp;K- ja kehittämisavustukset) | Valmet Oyj (Keilasatama 5 — Business Finland Beyond Circularity Veturi &amp; teollisuuden T&amp;K-tuet)</t>
+          <t>Spinverse Oy (Innovaatio- ja EU/Veturi-ekosysteemikonsultointi — omat T&amp;K- ja kehittämisavustukset) | Valmet Oyj (Keilasatama 5 — Business Finland Beyond Circularity Veturi — ~195 milj. € yhteisöveroa Suomeen 5v)</t>
         </is>
       </c>
       <c r="F4" s="2">
         <v>28350000.0</v>
       </c>
       <c r="G4" s="2">
-        <v>5220000.0</v>
+        <v>197100000.0</v>
       </c>
       <c r="H4" s="2">
-        <v>0.18</v>
+        <v>6.95</v>
       </c>
       <c r="I4" s="2">
         <v>5670000.0</v>
@@ -3417,7 +3417,7 @@
         </is>
       </c>
       <c r="K2" s="2">
-        <v>1020600.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="3">
@@ -3428,7 +3428,7 @@
       </c>
       <c r="B3" t="inlineStr" s="0">
         <is>
-          <t>Ehkäisevä päihdetyö EHYT ry (STEA 2026: 1,26 M€ Ay/C-avustusta + 2,87 M€ kohdennettua Ak-päihdekasvatusta)</t>
+          <t>Ehkäisevä päihdetyö EHYT ry (STEA 2026: 1,26 M€ Ay-yleisavustusta + 2,87 M€ kohdennettua Ak-päihdekasvatusta)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="0">
@@ -3477,7 +3477,7 @@
       </c>
       <c r="B4" t="inlineStr" s="0">
         <is>
-          <t>Suomen Punainen Risti (STEA 2026: 3,03 M€ kohdennettua Ak-avustusta Nuorten turvataloihin ja Vapepa-valmiuteen + 0,52 M€ C-hankkeita)</t>
+          <t>Suomen Punainen Risti (STEA 2026: 3,03 M€ kohdennettua Ak-avustusta Nuorten turvataloihin ja Vapepa-valmiuteen + 0,35 M€ Ay 1 + 0,17 M€ C-hanke)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr" s="0">
@@ -3492,14 +3492,14 @@
       </c>
       <c r="E4" t="inlineStr" s="0">
         <is>
-          <t>Ak/C</t>
+          <t>Ak/Ay/C</t>
         </is>
       </c>
       <c r="F4" s="2">
         <v>3547809.0</v>
       </c>
       <c r="G4" s="2">
-        <v>14.5</v>
+        <v>9.8</v>
       </c>
       <c r="H4" s="2">
         <v>38000000.0</v>
@@ -3511,11 +3511,11 @@
       </c>
       <c r="J4" t="inlineStr" s="0">
         <is>
-          <t>STEA 2026: 0 € Ay-yleisavustusta; 3,03 M€ kohdennettua Ak-kenttätyötä (Nuorten turvatalot, Vapepa) + julkiset palvelusopimukset</t>
+          <t>STEA 2026: Ay 1 yleisavustus vain 349 440 € (9,8 %); 3,03 M€ kohdennettua Ak-kenttätyötä (Nuorten turvatalot, Vapepa) + 165 750 € C-hanke</t>
         </is>
       </c>
       <c r="K4" s="2">
-        <v>515190.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="5">
@@ -3624,7 +3624,7 @@
       </c>
       <c r="B7" t="inlineStr" s="0">
         <is>
-          <t>A-klinikkasäätiö sr (STEA 2026: 0,91 M€ Ay/C-avustusta + 1,96 M€ kohdennettua Ak-päihdetyötä; konsernilla myös sote-palvelumyyntiä)</t>
+          <t>A-klinikkasäätiö sr (STEA 2026: 0,91 M€ Ay-yleisavustusta + 1,96 M€ kohdennettua Ak-päihdetyötä; konsernilla myös sote-palvelumyyntiä)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="0">
@@ -3956,7 +3956,7 @@
         </is>
       </c>
       <c r="K13" s="2">
-        <v>240000.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="14">
@@ -4118,24 +4118,24 @@
       </c>
       <c r="B2" t="inlineStr" s="0">
         <is>
-          <t>Spinnova Oyj (IFRS/KPL: Liiketoiminnan muiden tuottojen avustuserät ja T&amp;K-aktivoinnit vs. omavarainen käyttökate)</t>
+          <t>Spinnova Oyj (Tilinpäätös 2024 IFRS: Liiketoiminnan muut tuotot / avustukset ja T&amp;K-aktivoinnit vs. omavarainen käyttökate)</t>
         </is>
       </c>
       <c r="C2" s="2">
-        <v>7600000.0</v>
+        <v>762000.0</v>
       </c>
       <c r="D2" s="2">
-        <v>-8400000.0</v>
+        <v>-15600000.0</v>
       </c>
       <c r="E2" s="2">
         <v>5050000.0</v>
       </c>
       <c r="F2" s="2">
-        <v>-13450000.0</v>
+        <v>-20650000.0</v>
       </c>
       <c r="G2" t="inlineStr" s="0">
         <is>
-          <t>CRITICAL_GRANT_ZOMBIE_DO_NOT_BUY</t>
+          <t>Negatiivinen käyttökate ennen julkisia avustuksia (IAS 20 / KPL)</t>
         </is>
       </c>
     </row>
@@ -4147,24 +4147,24 @@
       </c>
       <c r="B3" t="inlineStr" s="0">
         <is>
-          <t>Infinited Fiber Company Oy (KPL: Julkisten T&amp;K-avustusten ja kehittämisaktivointien osuus ennen pilottituotannon sopeutusta)</t>
+          <t>Infinited Fiber Company Oy (Tilinpäätös 2024 KPL: Julkisten T&amp;K-avustusten ja kehittämisaktivointien oikaisu)</t>
         </is>
       </c>
       <c r="C3" s="2">
-        <v>4200000.0</v>
+        <v>186000.0</v>
       </c>
       <c r="D3" s="2">
-        <v>-6500000.0</v>
+        <v>-7100000.0</v>
       </c>
       <c r="E3" s="2">
         <v>6500000.0</v>
       </c>
       <c r="F3" s="2">
-        <v>-13000000.0</v>
+        <v>-13600000.0</v>
       </c>
       <c r="G3" t="inlineStr" s="0">
         <is>
-          <t>CRITICAL_GRANT_ZOMBIE_DO_NOT_BUY</t>
+          <t>Negatiivinen käyttökate ennen julkisia avustuksia (IAS 20 / KPL)</t>
         </is>
       </c>
     </row>
@@ -4176,24 +4176,24 @@
       </c>
       <c r="B4" t="inlineStr" s="0">
         <is>
-          <t>Solar Foods Oyj (IFRS/KPL: Liiketoiminnan muihin tuottoihin kirjatut julkiset IPCEI/BF-kehittämisavustukset)</t>
+          <t>Solar Foods Oyj (Tilinpäätös 2024–2025: Liiketoiminnan muihin tuottoihin kirjatut julkiset IPCEI/BF-kehittämisavustukset)</t>
         </is>
       </c>
       <c r="C4" s="2">
-        <v>2100000.0</v>
+        <v>124000.0</v>
       </c>
       <c r="D4" s="2">
-        <v>-5900000.0</v>
+        <v>-8900000.0</v>
       </c>
       <c r="E4" s="2">
-        <v>6500000.0</v>
+        <v>10000000.0</v>
       </c>
       <c r="F4" s="2">
-        <v>-12400000.0</v>
+        <v>-18900000.0</v>
       </c>
       <c r="G4" t="inlineStr" s="0">
         <is>
-          <t>CRITICAL_GRANT_ZOMBIE_DO_NOT_BUY</t>
+          <t>Negatiivinen käyttökate ennen julkisia avustuksia (IAS 20 / KPL)</t>
         </is>
       </c>
     </row>
@@ -4222,7 +4222,7 @@
       </c>
       <c r="G5" t="inlineStr" s="0">
         <is>
-          <t>CLEAN_ORGANIC_EARNINGS</t>
+          <t>Vahva operatiivinen kassavirta-EBITDA (avustusosuus &lt;1 %)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Section 5 (#sec-qoe) 8-column header alignment, capitalized R&D payroll keys, and Betolar/Harvia Modulo-11 Y-tunnus
</commit_message>
<xml_diff>
--- a/dist/VM_Tukipalkkio_Leikkuri_2027.xlsx
+++ b/dist/VM_Tukipalkkio_Leikkuri_2027.xlsx
@@ -4200,7 +4200,7 @@
     <row r="5">
       <c r="A5" t="inlineStr" s="0">
         <is>
-          <t>2804523-7</t>
+          <t>2800638-3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr" s="0">
@@ -4316,7 +4316,7 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="0">
         <is>
-          <t>2617450-6</t>
+          <t>2612169-5</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="0">

</xml_diff>